<commit_message>
Testing lab: threshold note, transcribed-run label, peer feedback
- tests/test_live.py: comment records that the 120 s first-response
  limit was set before the first run (not tuned to the 71.5 s result).
- live_history.jsonl: the 71.5 s run is labelled as manually transcribed.
- Peer feedback sheet/section: PF-1 (prior records from other
  hospitals/PCPs) out of scope - no such data, would need EHR
  integration - listed as future work; blank rows for further feedback.
- Report regenerated (161 passed; 20/20 test cases pass).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testing/test_cases.xlsx
+++ b/testing/test_cases.xlsx
@@ -10,13 +10,15 @@
     <sheet name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Defects" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Corrected tests" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Run summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Peer feedback" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Run summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test cases'!$A$1:$J$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Defects'!$A$1:$G$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Corrected tests'!$A$1:$E$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Run summary'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Peer feedback'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Run summary'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1381,7 +1383,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 test runs passed; all assertions in the expected result held. Measured: 50 requests, server memory 209.4 MB after startup, peak 214.4 MB (limit 512); latency median 40.3 ms, p95 63.5 ms, max 79.0 ms (limit p95 2000 ms); startup 3.39 s.</t>
+          <t>1 of 1 test runs passed; all assertions in the expected result held. Measured: 50 requests, server memory 209.8 MB after startup, peak 214.7 MB (limit 512); latency median 32.6 ms, p95 48.0 ms, max 60.7 ms (limit p95 2000 ms); startup 4.47 s.</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1433,7 +1435,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>1 of 1 test runs passed; all assertions in the expected result held. Latest run (2026-10-19T16:18:45+00:00): first response 0.4 s (service was already awake); warm /predict 0.2, 0.21, 0.22 s; /explain 0.25 s. All runs: 2026-10-19T16:13:46+00:00 first 71.47 s (asleep); 2026-10-19T16:17:20+00:00 first 0.2 s (awake); 2026-10-19T16:18:45+00:00 first 0.4 s (awake).</t>
+          <t>1 of 1 test runs passed; all assertions in the expected result held. Latest run (2026-10-19T16:29:30+00:00): first response 0.35 s (service was already awake); warm /predict 0.18, 0.21, 0.2 s; /explain 0.23 s. All runs: 2026-10-19T16:13:46+00:00 first 71.47 s (asleep) [manually transcribed]; 2026-10-19T16:17:20+00:00 first 0.2 s (awake); 2026-10-19T16:18:45+00:00 first 0.4 s (awake); 2026-10-19T16:29:30+00:00 first 0.35 s (awake).</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -2472,6 +2474,153 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Suggestion</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Rationale</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>PF-1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Peer review</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Incorporate prior records from other hospitals and primary care providers (PCPs).</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Out of scope</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>The UCI dataset has no records from other hospitals or PCPs, and getting them would need EHR integration and data-access agreements, which the Lab 4 requirements exclude for this one-semester proof of concept.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Listed as future work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>PF-2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>PF-3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>PF-4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>PF-5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>PF-6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2499,7 +2648,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19 11:19</t>
+          <t>2026-10-19 11:30</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2660,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>4cc8b16 (plus uncommitted changes)</t>
+          <t>006986b (plus uncommitted changes)</t>
         </is>
       </c>
     </row>
@@ -2523,7 +2672,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>161 passed, 3 warnings in 42.79s</t>
+          <t>161 passed, 3 warnings in 59.04s</t>
         </is>
       </c>
     </row>

</xml_diff>